<commit_message>
btn open report excel
</commit_message>
<xml_diff>
--- a/BaoCaoTracking/BaoCao_Tracking_28-04-2026.xlsx
+++ b/BaoCaoTracking/BaoCao_Tracking_28-04-2026.xlsx
@@ -155,6 +155,21 @@
   </x:si>
   <x:si>
     <x:t>lưu file excel design mới</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Ca 1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Nguyễn Phi Học</x:t>
+  </x:si>
+  <x:si>
+    <x:t>00026796354</x:t>
+  </x:si>
+  <x:si>
+    <x:t>M02-01-C</x:t>
+  </x:si>
+  <x:si>
+    <x:t>uyển test</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -809,14 +824,14 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:J12"/>
+  <x:dimension ref="A1:J13"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="11" max="16384" width="9.140625" style="1" customWidth="1"/>
     <x:col min="1" max="1" width="16.710625" style="1" customWidth="1"/>
     <x:col min="2" max="2" width="7.424911" style="1" customWidth="1"/>
     <x:col min="3" max="3" width="32.996339" style="1" customWidth="1"/>
-    <x:col min="4" max="4" width="19.282054" style="1" customWidth="1"/>
+    <x:col min="4" max="4" width="20.996339" style="1" customWidth="1"/>
     <x:col min="5" max="5" width="24.710625" style="1" customWidth="1"/>
     <x:col min="6" max="6" width="19.424911" style="1" customWidth="1"/>
     <x:col min="7" max="7" width="27.139196" style="1" customWidth="1"/>
@@ -1103,35 +1118,67 @@
       </x:c>
     </x:row>
     <x:row r="12" spans="1:10">
-      <x:c r="A12" s="13" t="s">
+      <x:c r="A12" s="10" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="B12" s="14" t="s">
+      <x:c r="B12" s="11" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="C12" s="14" t="s">
+      <x:c r="C12" s="11" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="D12" s="14" t="s">
+      <x:c r="D12" s="11" t="s">
         <x:v>38</x:v>
       </x:c>
-      <x:c r="E12" s="14" t="s">
+      <x:c r="E12" s="11" t="s">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="F12" s="14" t="s">
+      <x:c r="F12" s="11" t="s">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="G12" s="14">
+      <x:c r="G12" s="11">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="H12" s="14" t="s">
+      <x:c r="H12" s="11" t="s">
         <x:v>45</x:v>
       </x:c>
-      <x:c r="I12" s="14">
+      <x:c r="I12" s="11">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="J12" s="15" t="s">
+      <x:c r="J12" s="12" t="s">
         <x:v>46</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" spans="1:10">
+      <x:c r="A13" s="13" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B13" s="14" t="s">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="C13" s="14" t="s">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="D13" s="14" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="E13" s="14" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="F13" s="14" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="G13" s="14">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H13" s="14" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="I13" s="14">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="J13" s="15" t="s">
+        <x:v>51</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Update search by SKU
</commit_message>
<xml_diff>
--- a/BaoCaoTracking/BaoCao_Tracking_28-04-2026.xlsx
+++ b/BaoCaoTracking/BaoCao_Tracking_28-04-2026.xlsx
@@ -170,6 +170,48 @@
   </x:si>
   <x:si>
     <x:t>uyển test</x:t>
+  </x:si>
+  <x:si>
+    <x:t>00002673</x:t>
+  </x:si>
+  <x:si>
+    <x:t>021*5</x:t>
+  </x:si>
+  <x:si>
+    <x:t>M05-03-D</x:t>
+  </x:si>
+  <x:si>
+    <x:t>M03-03-A, M05-02-D</x:t>
+  </x:si>
+  <x:si>
+    <x:t>test search sku *</x:t>
+  </x:si>
+  <x:si>
+    <x:t>0001696219</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1796*3</x:t>
+  </x:si>
+  <x:si>
+    <x:t>M02-04-A</x:t>
+  </x:si>
+  <x:si>
+    <x:t>test sku</x:t>
+  </x:si>
+  <x:si>
+    <x:t>0002691456</x:t>
+  </x:si>
+  <x:si>
+    <x:t>sku lưu *</x:t>
+  </x:si>
+  <x:si>
+    <x:t>000000000</x:t>
+  </x:si>
+  <x:si>
+    <x:t>M05-04-B</x:t>
+  </x:si>
+  <x:si>
+    <x:t>**</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -824,7 +866,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:J13"/>
+  <x:dimension ref="A1:J17"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="11" max="16384" width="9.140625" style="1" customWidth="1"/>
@@ -1150,35 +1192,163 @@
       </x:c>
     </x:row>
     <x:row r="13" spans="1:10">
-      <x:c r="A13" s="13" t="s">
+      <x:c r="A13" s="10" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="B13" s="14" t="s">
+      <x:c r="B13" s="11" t="s">
         <x:v>47</x:v>
       </x:c>
-      <x:c r="C13" s="14" t="s">
+      <x:c r="C13" s="11" t="s">
         <x:v>48</x:v>
       </x:c>
-      <x:c r="D13" s="14" t="s">
+      <x:c r="D13" s="11" t="s">
         <x:v>49</x:v>
       </x:c>
-      <x:c r="E13" s="14" t="s">
+      <x:c r="E13" s="11" t="s">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="F13" s="14" t="s">
+      <x:c r="F13" s="11" t="s">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="G13" s="14">
+      <x:c r="G13" s="11">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="H13" s="14" t="s">
+      <x:c r="H13" s="11" t="s">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="I13" s="14">
+      <x:c r="I13" s="11">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="J13" s="15" t="s">
+      <x:c r="J13" s="12" t="s">
         <x:v>51</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" spans="1:10">
+      <x:c r="A14" s="10" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B14" s="11" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C14" s="11" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="D14" s="11" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="E14" s="11" t="s">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="F14" s="11" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="G14" s="11">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H14" s="11" t="s">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="I14" s="11">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J14" s="12" t="s">
+        <x:v>56</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" spans="1:10">
+      <x:c r="A15" s="10" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B15" s="11" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C15" s="11" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="D15" s="11" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="E15" s="11" t="s">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="F15" s="11" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="G15" s="11">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H15" s="11" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="I15" s="11">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="J15" s="12" t="s">
+        <x:v>60</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" spans="1:10">
+      <x:c r="A16" s="10" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B16" s="11" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C16" s="11" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="D16" s="11" t="s">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="E16" s="11" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="F16" s="11" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="G16" s="11">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H16" s="11" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="I16" s="11">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J16" s="12" t="s">
+        <x:v>62</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" spans="1:10">
+      <x:c r="A17" s="13" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B17" s="14" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C17" s="14" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="D17" s="14" t="s">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="E17" s="14" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="F17" s="14" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="G17" s="14">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H17" s="14" t="s">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="I17" s="14">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J17" s="15" t="s">
+        <x:v>65</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>